<commit_message>
Frais de port : paliers relevés sur les colis lourds / paniers multiples (jamais de perte), + fichier Excel de référence à jour
</commit_message>
<xml_diff>
--- a/docs/Niv-Creation-Prix-et-Port.xlsx
+++ b/docs/Niv-Creation-Prix-et-Port.xlsx
@@ -878,11 +878,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -938,172 +938,227 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>de 2 à 5 kg</t>
+          <t>de 2 à 3 kg</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>6,90 €</t>
+          <t>7,50 €</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>plus de 5 kg</t>
+          <t>de 3 à 5 kg</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>8,90 €</t>
+          <t>8,50 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>de 5 à 10 kg</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>9,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>de 10 à 15 kg</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>12,90 €</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>plus de 15 kg</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>15,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>DOMICILE (Colissimo) — par poids</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Poids du colis</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Prix</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>jusqu'à 1 kg</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>6,90 €</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>de 1 à 2 kg</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>8,90 €</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>de 2 à 5 kg</t>
+          <t>jusqu'à 1 kg</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>14,90 €</t>
+          <t>6,90 €</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>de 5 à 10 kg</t>
+          <t>de 1 à 2 kg</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>22,90 €</t>
+          <t>8,90 €</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>plus de 10 kg</t>
+          <t>de 2 à 5 kg</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>29,90 €</t>
+          <t>14,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>de 5 à 10 kg</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>22,90 €</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>de 10 à 15 kg</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>28,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>plus de 15 kg</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>34,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>DOMICILE — par quantité (petits produits)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Paliers</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Déco (bois)</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>1 à 4 : 6,90 €  ·  5 à 12 : 12,90 €  ·  13+ : 19,90 €</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>Verres (fragiles)</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>1 à 2 : 11,90 €  ·  3 à 4 : 16,90 €  ·  5+ : 21,90 €</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Bijoux / petits objets</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Lettre suivie : 3,90 € (offert dès 45 €)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>RÈGLE : domicile = le PLUS ÉLEVÉ entre le tarif « par quantité » et le tarif « par poids » → jamais sous-facturé, et les petits produits ne changent pas.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Point relais = ton mode principal (le plus doux). Retrait en main propre (déco/mariage, zone 95 + voisins) = gratuit.</t>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Point relais = ton mode principal (le plus doux). Paliers relevés le 06/07/2026 pour ne jamais perdre d'argent sur les paniers lourds/à plusieurs objets, tout en restant dans les prix du marché.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Retrait en main propre (déco/mariage, zone 95 + voisins) = gratuit.</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1359,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>6,90 €</t>
+          <t>7,50 €</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1326,7 +1381,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>6,90 €</t>
+          <t>8,50 €</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1348,7 +1403,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>8,90 €</t>
+          <t>9,90 €</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1370,7 +1425,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>8,90 €</t>
+          <t>9,90 €</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1392,7 +1447,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>6,90 €</t>
+          <t>8,50 €</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1414,7 +1469,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>6,90 €</t>
+          <t>7,50 €</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Doc Excel : ajout exemples paniers lourds (4 XL, 4 XL + socles, 6 XL)
</commit_message>
<xml_diff>
--- a/docs/Niv-Creation-Prix-et-Port.xlsx
+++ b/docs/Niv-Creation-Prix-et-Port.xlsx
@@ -1264,7 +1264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1437,64 +1437,130 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Petit + Moyen + Grand</t>
+          <t>4 blocs XL</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>3,65 kg</t>
+          <t>11,20 kg</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>8,50 €</t>
+          <t>12,90 €</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>14,90 €</t>
+          <t>28,90 €</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>1 bijou + 1 bloc XL</t>
+          <t>4 blocs XL + 4 socles</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>2,84 kg</t>
+          <t>13,40 kg</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>7,50 €</t>
+          <t>12,90 €</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>14,90 €</t>
+          <t>28,90 €</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>6 blocs XL</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>16,80 kg</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>15,90 €</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>34,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Petit + Moyen + Grand</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>3,65 kg</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>8,50 €</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>14,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>1 bijou + 1 bloc XL</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>2,84 kg</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>7,50 €</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>14,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t>1 bijou seul</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>0,04 kg</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>4,90 €</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>3,90 €</t>
         </is>

</xml_diff>

<commit_message>
Livraison Europe : tarifs par zone (EU1/EU2/Suisse) + poids, sélecteur pays au panier, adresse verrouillée sur le pays choisi (France inchangée)
</commit_message>
<xml_diff>
--- a/docs/Niv-Creation-Prix-et-Port.xlsx
+++ b/docs/Niv-Creation-Prix-et-Port.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Comment ça se calcule" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Exemples" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Ajouter un produit" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Livraison Europe" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1660,4 +1661,405 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LIVRAISON EUROPE (hors France) — par zone &amp; par poids</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>France + Monaco = tarifs habituels (onglet Frais de port). Ci-dessous : les autres pays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>ZONE EU1 — Belgique · Luxembourg · Pays-Bas · Allemagne</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Type / poids</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Prix</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Bijou / petit objet (lettre) ≤ 250 g</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>6,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Bijou (lettre) ≤ 500 g</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>9,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Bijou (lettre) ≤ 2 kg</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>12,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Colis ≤ 1 kg</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>16,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Colis ≤ 2 kg</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>22,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Colis ≤ 5 kg</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>32,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Colis ≤ 10 kg</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>46,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Colis + 10 kg</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>74,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>ZONE EU2 — Espagne · Italie · Portugal</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Type / poids</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Prix</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Bijou (lettre) ≤ 250 g</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>7,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Bijou (lettre) ≤ 500 g</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>10,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Bijou (lettre) ≤ 2 kg</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>14,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Colis ≤ 1 kg</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>18,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Colis ≤ 2 kg</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>24,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Colis ≤ 5 kg</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>36,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Colis ≤ 10 kg</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>52,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Colis + 10 kg</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>84,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>ZONE SUISSE (hors UE : douane, plus cher)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Type / poids</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Prix</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Bijou (lettre) ≤ 250 g</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>8,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Bijou (lettre) ≤ 500 g</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>12,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Bijou (lettre) ≤ 2 kg</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>17,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Colis ≤ 1 kg</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>22,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>Colis ≤ 2 kg</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>29,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Colis ≤ 5 kg</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>44,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>Colis ≤ 10 kg</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>64,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Colis + 10 kg</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>99,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>• Europe = livraison à domicile uniquement (Colissimo / lettre suivie internationale). Point relais Europe = possible plus tard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>• Le client choisit son pays sur la page panier ; le tarif exact s'affiche au paiement. Tarifs au-dessus du coût réel → aucune perte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>• Exemples : 1 bijou vers Belgique = 6,90 € · 1 bloc XL vers Belgique = 32,90 € · vers Espagne = 36,90 € · vers Suisse = 44,90 €.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Point relais multi-transporteurs : Mondial Relay, Relais Colis, Colissimo, Chrono Shop2Shop, UPS — tous les points sur la carte, prix par transporteur au poids (Boxtal)
</commit_message>
<xml_diff>
--- a/docs/Niv-Creation-Prix-et-Port.xlsx
+++ b/docs/Niv-Creation-Prix-et-Port.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Exemples" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Ajouter un produit" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Livraison Europe" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Transporteurs relais" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2062,4 +2063,249 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>POINT RELAIS — plusieurs transporteurs (le client choisit sur la carte)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Le client voit TOUS les points relais autour de lui (tous transporteurs) et clique sur le plus proche. Le prix s'ajuste au transporteur du point choisi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Transporteur</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>≤ 1 kg</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>≤ 2 kg</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>≤ 5 kg</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>≤ 10 kg</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>+ 10 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Mondial Relay</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>4,90 €</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>6,50 €</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>8,50 €</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>9,90 €</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>15,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Relais Colis</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>5,50 €</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>6,90 €</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>8,90 €</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>10,90 €</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>16,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Colissimo (La Poste)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>5,50 €</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>7,50 €</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>10,90 €</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>15,90 €</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>25,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Chrono Shop2Shop</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>5,90 €</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>7,50 €</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>9,90 €</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>12,90 €</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>16,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>UPS Point Relais</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>6,90 €</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>8,90 €</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>12,90 €</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>17,90 €</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>24,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>• Tous ces transporteurs sont gérés par Boxtal (compte inscrit). Mondial Relay = le moins cher. Tarifs au-dessus du coût réel → aucune perte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>• Pour ajouter/retirer un transporteur : liste RELAIS_CARRIERS dans src/lib/shipping.js (il doit aussi être activé sur Boxtal).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Doc Excel : point relais Europe (EU1/EU2) ajouté à l'onglet Livraison Europe
</commit_message>
<xml_diff>
--- a/docs/Niv-Creation-Prix-et-Port.xlsx
+++ b/docs/Niv-Creation-Prix-et-Port.xlsx
@@ -1670,7 +1670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2037,23 +2037,145 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>• Europe = livraison à domicile uniquement (Colissimo / lettre suivie internationale). Point relais Europe = possible plus tard.</t>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>POINT RELAIS EUROPE (Mondial Relay) — Belgique · Luxembourg · Pays-Bas · Espagne · Italie · Portugal</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>• Le client choisit son pays sur la page panier ; le tarif exact s'affiche au paiement. Tarifs au-dessus du coût réel → aucune perte.</t>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Zone / poids</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Prix</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>• Exemples : 1 bijou vers Belgique = 6,90 € · 1 bloc XL vers Belgique = 32,90 € · vers Espagne = 36,90 € · vers Suisse = 44,90 €.</t>
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>EU1 (BE/LU/NL) — ≤ 1 kg</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>9,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>EU1 — ≤ 2 kg</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>11,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>EU1 — ≤ 5 kg</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>16,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>EU1 — ≤ 10 kg</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>22,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>EU2 (ES/IT/PT) — ≤ 1 kg</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>11,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>EU2 — ≤ 2 kg</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>13,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>EU2 — ≤ 5 kg</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>19,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>EU2 — ≤ 10 kg</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>26,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>• Allemagne &amp; Suisse : PAS de point relais → livraison à domicile uniquement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>• Le client choisit son pays sur la page panier ; à domicile ou point relais (où dispo). Tarifs au-dessus du coût réel → aucune perte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>• Exemples domicile : 1 bijou vers Belgique = 6,90 € · 1 bloc XL vers Belgique = 32,90 € · Espagne = 36,90 € · Suisse = 44,90 €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>• Exemples point relais : 1 bloc XL vers Belgique = 16,90 € · vers Espagne = 19,90 € (bien moins cher que le domicile).</t>
         </is>
       </c>
     </row>

</xml_diff>